<commit_message>
Atualiza dados - 07/08/2026  9:38
</commit_message>
<xml_diff>
--- a/fpse/CAF.xlsx
+++ b/fpse/CAF.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fpse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82F8FCD-45E2-436E-82FB-A35293DF1F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F96909-2C82-4A40-A9C0-C0D6D1E5625B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cenários homologação" sheetId="6" r:id="rId1"/>
@@ -852,7 +852,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -885,6 +885,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1199,7 +1203,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1243,7 +1246,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>215</v>
       </c>
@@ -1274,7 +1277,7 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>215</v>
       </c>
@@ -1305,7 +1308,7 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>215</v>
       </c>
@@ -1336,7 +1339,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>215</v>
       </c>
@@ -1367,7 +1370,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>215</v>
       </c>
@@ -1398,7 +1401,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>210</v>
       </c>
@@ -1429,7 +1432,7 @@
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>211</v>
       </c>
@@ -1460,7 +1463,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>208</v>
       </c>
@@ -1491,7 +1494,7 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>211</v>
       </c>
@@ -1522,7 +1525,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>208</v>
       </c>
@@ -1553,7 +1556,7 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>208</v>
       </c>
@@ -1584,7 +1587,7 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>215</v>
       </c>
@@ -1615,7 +1618,7 @@
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>210</v>
       </c>
@@ -1646,7 +1649,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>211</v>
       </c>
@@ -1677,7 +1680,7 @@
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>215</v>
       </c>
@@ -1708,7 +1711,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>215</v>
       </c>
@@ -1770,7 +1773,7 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>215</v>
       </c>
@@ -1801,7 +1804,7 @@
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>215</v>
       </c>
@@ -1832,7 +1835,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>215</v>
       </c>
@@ -1863,7 +1866,7 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>215</v>
       </c>
@@ -1894,7 +1897,7 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>215</v>
       </c>
@@ -1925,7 +1928,7 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>215</v>
       </c>
@@ -1987,7 +1990,7 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>215</v>
       </c>
@@ -2018,7 +2021,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>215</v>
       </c>
@@ -2049,7 +2052,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>215</v>
       </c>
@@ -2083,7 +2086,7 @@
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>131</v>
@@ -2109,7 +2112,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>213</v>
       </c>
@@ -2140,7 +2143,7 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>215</v>
       </c>
@@ -2171,7 +2174,7 @@
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>210</v>
       </c>
@@ -2202,7 +2205,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>210</v>
       </c>
@@ -2233,7 +2236,7 @@
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>210</v>
       </c>
@@ -2264,7 +2267,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>215</v>
       </c>
@@ -2295,7 +2298,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>215</v>
       </c>
@@ -2326,7 +2329,7 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>215</v>
       </c>
@@ -2357,7 +2360,7 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>215</v>
       </c>
@@ -2388,7 +2391,7 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
         <v>200</v>
@@ -2449,7 +2452,7 @@
     <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>176</v>
@@ -2535,7 +2538,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>208</v>
       </c>
@@ -2567,15 +2570,7 @@
       <c r="K44" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Aguadando cenários"/>
-        <filter val="Disponivel para Reteste"/>
-        <filter val="Em Correção"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2754,7 +2749,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E94EB92-949A-4861-8A92-72A5C32EFB43}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.77734375" customWidth="1"/>
@@ -2894,7 +2889,7 @@
         <v>5</v>
       </c>
       <c r="J4" s="12">
-        <f t="shared" ref="J4:J10" si="0">C4+D4+E4+F4+G4+H4+I4</f>
+        <f t="shared" ref="J4:J11" si="0">C4+D4+E4+F4+G4+H4+I4</f>
         <v>38</v>
       </c>
     </row>
@@ -3086,14 +3081,47 @@
         <v>15</v>
       </c>
       <c r="H10" s="16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10" s="16">
         <v>0</v>
       </c>
       <c r="J10" s="17">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="14">
+        <v>0.375</v>
+      </c>
+      <c r="B11" s="15">
+        <v>46241</v>
+      </c>
+      <c r="C11" s="18">
+        <v>0</v>
+      </c>
+      <c r="D11" s="18">
+        <v>2</v>
+      </c>
+      <c r="E11" s="18">
+        <v>0</v>
+      </c>
+      <c r="F11" s="18">
+        <v>20</v>
+      </c>
+      <c r="G11" s="18">
+        <v>15</v>
+      </c>
+      <c r="H11" s="18">
+        <v>1</v>
+      </c>
+      <c r="I11" s="18">
+        <v>0</v>
+      </c>
+      <c r="J11" s="19">
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados - 07/08/2026 16:06
</commit_message>
<xml_diff>
--- a/fpse/CAF.xlsx
+++ b/fpse/CAF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiago.delima\painel_hml_caf\fpse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F96909-2C82-4A40-A9C0-C0D6D1E5625B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92666BBF-9E2E-492E-B54D-9A75CA3F2755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -852,7 +852,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -885,10 +885,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1203,6 +1199,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1246,7 +1243,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>215</v>
       </c>
@@ -1277,12 +1274,12 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>215</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>16</v>
@@ -1308,12 +1305,12 @@
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>215</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>23</v>
@@ -1339,12 +1336,12 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>215</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>28</v>
@@ -1370,7 +1367,7 @@
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>215</v>
       </c>
@@ -1432,12 +1429,12 @@
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>211</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>43</v>
@@ -1463,7 +1460,7 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>208</v>
       </c>
@@ -1494,7 +1491,7 @@
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>211</v>
       </c>
@@ -1525,7 +1522,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>208</v>
       </c>
@@ -1556,7 +1553,7 @@
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>208</v>
       </c>
@@ -1587,7 +1584,7 @@
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>215</v>
       </c>
@@ -1649,7 +1646,7 @@
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>211</v>
       </c>
@@ -1680,7 +1677,7 @@
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>215</v>
       </c>
@@ -1711,7 +1708,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>215</v>
       </c>
@@ -1742,12 +1739,12 @@
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>215</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>88</v>
@@ -1773,7 +1770,7 @@
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>215</v>
       </c>
@@ -1835,7 +1832,7 @@
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>215</v>
       </c>
@@ -1866,7 +1863,7 @@
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>215</v>
       </c>
@@ -1897,7 +1894,7 @@
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>215</v>
       </c>
@@ -1928,7 +1925,7 @@
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>215</v>
       </c>
@@ -1959,7 +1956,7 @@
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>215</v>
       </c>
@@ -1990,7 +1987,7 @@
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>215</v>
       </c>
@@ -2021,7 +2018,7 @@
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>215</v>
       </c>
@@ -2052,7 +2049,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>215</v>
       </c>
@@ -2112,7 +2109,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>213</v>
       </c>
@@ -2143,7 +2140,7 @@
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>215</v>
       </c>
@@ -2267,7 +2264,7 @@
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>215</v>
       </c>
@@ -2298,7 +2295,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>215</v>
       </c>
@@ -2329,7 +2326,7 @@
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>215</v>
       </c>
@@ -2360,7 +2357,7 @@
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>215</v>
       </c>
@@ -2391,7 +2388,7 @@
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
         <v>200</v>
@@ -2420,7 +2417,7 @@
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4" t="s">
         <v>200</v>
@@ -2449,7 +2446,7 @@
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
     </row>
-    <row r="41" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="86.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
         <v>200</v>
@@ -2478,7 +2475,7 @@
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="4" t="s">
         <v>200</v>
@@ -2507,7 +2504,7 @@
       <c r="J42" s="6"/>
       <c r="K42" s="6"/>
     </row>
-    <row r="43" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="100.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>215</v>
       </c>
@@ -2538,7 +2535,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>208</v>
       </c>
@@ -2570,7 +2567,13 @@
       <c r="K44" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}"/>
+  <autoFilter ref="B1:B44" xr:uid="{C39B64EC-B305-411B-89CD-90AE48303B1A}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Cenário cancelado"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -3093,33 +3096,33 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
-        <v>0.375</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="B11" s="15">
         <v>46241</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="16">
         <v>0</v>
       </c>
-      <c r="D11" s="18">
-        <v>2</v>
-      </c>
-      <c r="E11" s="18">
+      <c r="D11" s="16">
         <v>0</v>
       </c>
-      <c r="F11" s="18">
-        <v>20</v>
-      </c>
-      <c r="G11" s="18">
-        <v>15</v>
-      </c>
-      <c r="H11" s="18">
+      <c r="E11" s="16">
         <v>1</v>
       </c>
-      <c r="I11" s="18">
+      <c r="F11" s="16">
+        <v>25</v>
+      </c>
+      <c r="G11" s="16">
+        <v>12</v>
+      </c>
+      <c r="H11" s="16">
         <v>0</v>
       </c>
-      <c r="J11" s="19">
+      <c r="I11" s="16">
+        <v>0</v>
+      </c>
+      <c r="J11" s="17">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>

</xml_diff>